<commit_message>
D-034 Step 2: add Seq_Status/Stimulus_VSL to VPR template, BALU VPR, and vplan_parser
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pssgen_vpr_template.xlsx
+++ b/docs/pssgen_vpr_template.xlsx
@@ -1095,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1155,6 +1155,168 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Seq_Status</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Stimulus_VSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
D-034 Step 5c: VSL authoring quality gates — VSL_Notes, Seq_Review, vsl_validator
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pssgen_vpr_template.xlsx
+++ b/docs/pssgen_vpr_template.xlsx
@@ -1095,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1165,6 +1165,16 @@
           <t>Stimulus_VSL</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>VSL_Notes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Seq_Review</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="J3" t="inlineStr">
@@ -1172,7 +1182,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="J4" t="inlineStr">
@@ -1180,7 +1195,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="J5" t="inlineStr">
@@ -1188,7 +1208,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="J6" t="inlineStr">
@@ -1196,7 +1221,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="J7" t="inlineStr">
@@ -1204,7 +1234,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="J8" t="inlineStr">
@@ -1212,7 +1247,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="J9" t="inlineStr">
@@ -1220,7 +1260,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="J10" t="inlineStr">
@@ -1228,7 +1273,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="J11" t="inlineStr">
@@ -1236,7 +1286,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="J12" t="inlineStr">
@@ -1244,7 +1299,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="J13" t="inlineStr">
@@ -1252,7 +1312,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="J14" t="inlineStr">
@@ -1260,7 +1325,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="J15" t="inlineStr">
@@ -1268,7 +1338,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="J16" t="inlineStr">
@@ -1276,7 +1351,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="J17" t="inlineStr">
@@ -1284,7 +1364,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="J18" t="inlineStr">
@@ -1292,7 +1377,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="J19" t="inlineStr">
@@ -1300,7 +1390,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="J20" t="inlineStr">
@@ -1308,7 +1403,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="J21" t="inlineStr">
@@ -1316,7 +1416,12 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
D-034 Step 5c follow-up: dropdown validation on Seq_Review/Seq_Status columns
Add openpyxl DataValidation dropdowns to col J (Seq_Status) and col M
(Seq_Review) rows 3-21 in both the BALU VPR and the VPR template.
Update balu_coverage_results.json: APPROVED=18, DRAFT=0, coverage_pct=94.74.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pssgen_vpr_template.xlsx
+++ b/docs/pssgen_vpr_template.xlsx
@@ -1182,7 +1182,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1195,7 +1194,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1208,7 +1206,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1221,7 +1218,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1234,7 +1230,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1247,7 +1242,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1260,7 +1254,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1273,7 +1266,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1286,7 +1278,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1299,7 +1290,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1312,7 +1302,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1325,7 +1314,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1338,7 +1326,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1351,7 +1338,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1364,7 +1350,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1377,7 +1362,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1390,7 +1374,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1403,7 +1386,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1416,7 +1398,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>DRAFT</t>
@@ -1427,12 +1408,18 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose from the list." promptTitle="COV Status" prompt="PLANNED / IMPLEMENTED / PASSING / FAILING" type="list">
       <formula1>"PLANNED,IMPLEMENTED,PASSING,FAILING"</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Functional,Code,Assertion,Toggle,FSM,Mixed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M3:M21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"DRAFT,REVIEWED,APPROVED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"NONE,PHASE_1,PHASE_2_GAP"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>